<commit_message>
feat(accounting): add UniGas client and four cars
Register شركة يونيغاز as an official client with plates 22219, 22084, 22076, and 22339 so those receipts route to DB_شركة_يونيغاز instead of unclassified.

Co-authored-by: lilly9reilly-dotcom <lilly9reilly-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/sheet-organization/قواعد_بيانات_العملاء.xlsx
+++ b/artifacts/sheet-organization/قواعد_بيانات_العملاء.xlsx
@@ -17,9 +17,10 @@
     <sheet name="DB_علي_صبار" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="DB_قيصر_شمري" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="DB_شركة" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="DB_غير_مصنف" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="2026_09" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="F_2026_09" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DB_شركة_يونيغاز" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DB_غير_مصنف" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026_09" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="F_2026_09" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -633,6 +634,28 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>DB_شركة</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DB_شركة_يونيغاز</t>
         </is>
       </c>
     </row>
@@ -887,6 +910,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الوصل</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>السائق</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>رقم السيارة</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>تاريخ التحميل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تاريخ التفريغ</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الكمية طن</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوجهة</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>نوع الحركة</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>الشهر</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>الفترة</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>سعر الطن</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>لترات الكاز</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>قيمة الكاز</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>المعتمد</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>وقت الترحيل</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>مفتاح الترحيل</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
@@ -983,7 +1126,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1085,7 +1228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2040,6 +2183,102 @@
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>22219</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>22084</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>22076</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>22339</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2051,7 +2290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2915,6 +3154,94 @@
       <c r="D39" t="inlineStr">
         <is>
           <t>DB_شركة</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>22219</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DB_شركة_يونيغاز</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>22084</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>DB_شركة_يونيغاز</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>22076</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>DB_شركة_يونيغاز</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>شركة يونيغاز</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>معتمد</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>22339</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DB_شركة_يونيغاز</t>
         </is>
       </c>
     </row>

</xml_diff>